<commit_message>
docs(diccionario_datos_customers): reorganize hyperlinks in data dictionary
</commit_message>
<xml_diff>
--- a/documents/diccionario_datos_customers.xlsx
+++ b/documents/diccionario_datos_customers.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jhayd\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jhayd\Documents\GitHub\jhayderstiven-Colab-03\customers\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D02F3BF-D6C7-471F-8381-718FAD016BAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{793247C4-D9CC-437C-9CBE-4F30A0A149E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DICCIONARIO DE DATOS " sheetId="2" r:id="rId1"/>
@@ -109,9 +109,6 @@
     <t>Catálogo de Datos - Información General</t>
   </si>
   <si>
-    <t>carlos Alberto Espinel Camargo</t>
-  </si>
-  <si>
     <t>Incluyen tablas auxiliares como DEPARTMENTS, SPECIALTIES, ROLES, PERMISSIONS, ROOM_TYPES, STATUS_CODES, las cuales proveen contexto adicional, reducen redundancia y fortalecen la coherencia del sistema.</t>
   </si>
   <si>
@@ -552,6 +549,9 @@
   </si>
   <si>
     <t>SHIPMENT_ORDERS!A1</t>
+  </si>
+  <si>
+    <t>Jhayder Stiven Florez Camacho</t>
   </si>
 </sst>
 </file>
@@ -982,6 +982,60 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -991,59 +1045,20 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1054,6 +1069,18 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1063,35 +1090,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1566,938 +1566,1005 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="32.4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="50" t="s">
-        <v>52</v>
-      </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="51"/>
+      <c r="A1" s="39" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="52" t="s">
-        <v>53</v>
-      </c>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
+      <c r="B3" s="42" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="42"/>
     </row>
     <row r="4" spans="1:8" ht="67.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="38" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="40"/>
+      <c r="B4" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="44"/>
+      <c r="G4" s="44"/>
+      <c r="H4" s="45"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="44" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="44"/>
+      <c r="B5" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:8" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="39"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
-      <c r="G6" s="39"/>
-      <c r="H6" s="40"/>
+      <c r="B6" s="43" t="s">
+        <v>166</v>
+      </c>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
+      <c r="H6" s="45"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="53">
-        <v>46115</v>
-      </c>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
-      <c r="G7" s="44"/>
-      <c r="H7" s="44"/>
+      <c r="B7" s="46">
+        <v>46126</v>
+      </c>
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="38"/>
+      <c r="G7" s="38"/>
+      <c r="H7" s="38"/>
     </row>
     <row r="8" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="44"/>
-      <c r="H8" s="44"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="38"/>
     </row>
     <row r="9" spans="1:8" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A9" s="48" t="s">
+      <c r="A9" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="48"/>
-      <c r="C9" s="48"/>
-      <c r="D9" s="48"/>
-      <c r="E9" s="48"/>
-      <c r="F9" s="48"/>
-      <c r="G9" s="48"/>
-      <c r="H9" s="48"/>
+      <c r="B9" s="41"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="41"/>
+      <c r="H9" s="41"/>
     </row>
     <row r="10" spans="1:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="44" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
+      <c r="B10" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="38"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="38"/>
     </row>
     <row r="11" spans="1:8" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="44" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="44"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
-      <c r="G11" s="44"/>
-      <c r="H11" s="44"/>
+      <c r="B11" s="38" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="38"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="38"/>
+      <c r="F11" s="38"/>
+      <c r="G11" s="38"/>
+      <c r="H11" s="38"/>
     </row>
     <row r="12" spans="1:8" ht="66.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="44" t="s">
-        <v>57</v>
-      </c>
-      <c r="C12" s="44"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
-      <c r="H12" s="44"/>
+      <c r="B12" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="38"/>
     </row>
     <row r="13" spans="1:8" ht="52.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="44" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" s="44"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-      <c r="G13" s="44"/>
-      <c r="H13" s="44"/>
+      <c r="B13" s="38" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="38"/>
     </row>
     <row r="14" spans="1:8" ht="62.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="44" t="s">
-        <v>59</v>
-      </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="44"/>
-      <c r="H14" s="44"/>
+      <c r="B14" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="38"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="38"/>
     </row>
     <row r="15" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="44" t="s">
-        <v>60</v>
-      </c>
-      <c r="C15" s="44"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="44"/>
-      <c r="F15" s="44"/>
-      <c r="G15" s="44"/>
-      <c r="H15" s="44"/>
+      <c r="B15" s="38" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="38"/>
+      <c r="H15" s="38"/>
     </row>
     <row r="16" spans="1:8" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A16" s="48" t="s">
+      <c r="A16" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="48"/>
-      <c r="C16" s="48"/>
-      <c r="D16" s="48"/>
-      <c r="E16" s="48"/>
-      <c r="F16" s="48"/>
-      <c r="G16" s="48"/>
-      <c r="H16" s="48"/>
+      <c r="B16" s="41"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="41"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="41"/>
+      <c r="H16" s="41"/>
     </row>
     <row r="17" spans="1:8" ht="18" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="49" t="s">
+      <c r="B17" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="49"/>
-      <c r="D17" s="49"/>
-      <c r="E17" s="49"/>
-      <c r="F17" s="49" t="s">
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="47"/>
+      <c r="F17" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="G17" s="49"/>
-      <c r="H17" s="49"/>
+      <c r="G17" s="47"/>
+      <c r="H17" s="47"/>
     </row>
     <row r="18" spans="1:8" ht="96.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" s="38" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="44" t="s">
-        <v>62</v>
-      </c>
-      <c r="C18" s="44"/>
-      <c r="D18" s="44"/>
-      <c r="E18" s="44"/>
-      <c r="F18" s="45" t="str">
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="49" t="str">
         <f>CONCATENATE(A18,"_LINK")</f>
         <v>CUSTOMERS_LINK</v>
       </c>
-      <c r="G18" s="45"/>
-      <c r="H18" s="45"/>
+      <c r="G18" s="49"/>
+      <c r="H18" s="49"/>
     </row>
     <row r="19" spans="1:8" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B19" s="38" t="s">
         <v>83</v>
       </c>
-      <c r="B19" s="44" t="s">
-        <v>84</v>
-      </c>
-      <c r="C19" s="44"/>
-      <c r="D19" s="44"/>
-      <c r="E19" s="44"/>
-      <c r="F19" s="41" t="str">
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="50" t="str">
         <f t="shared" ref="F19" si="0">$F$18</f>
         <v>CUSTOMERS_LINK</v>
       </c>
-      <c r="G19" s="42"/>
-      <c r="H19" s="43"/>
+      <c r="G19" s="51"/>
+      <c r="H19" s="52"/>
     </row>
     <row r="20" spans="1:8" ht="56.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="38" t="s">
         <v>100</v>
       </c>
-      <c r="B20" s="44" t="s">
-        <v>101</v>
-      </c>
-      <c r="C20" s="44"/>
-      <c r="D20" s="44"/>
-      <c r="E20" s="44"/>
-      <c r="F20" s="47" t="str">
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="53" t="str">
         <f t="shared" ref="F20" si="1">$F$19</f>
         <v>CUSTOMERS_LINK</v>
       </c>
-      <c r="G20" s="47"/>
-      <c r="H20" s="47"/>
+      <c r="G20" s="53"/>
+      <c r="H20" s="53"/>
     </row>
     <row r="21" spans="1:8" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B21" s="38" t="s">
         <v>103</v>
       </c>
-      <c r="B21" s="44" t="s">
-        <v>104</v>
-      </c>
-      <c r="C21" s="44"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="44"/>
-      <c r="F21" s="46" t="s">
-        <v>109</v>
-      </c>
-      <c r="G21" s="46"/>
-      <c r="H21" s="46"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="48" t="s">
+        <v>108</v>
+      </c>
+      <c r="G21" s="48"/>
+      <c r="H21" s="48"/>
     </row>
     <row r="22" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B22" s="44" t="s">
-        <v>110</v>
-      </c>
-      <c r="C22" s="44"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="44"/>
-      <c r="F22" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="G22" s="45"/>
-      <c r="H22" s="45"/>
+        <v>72</v>
+      </c>
+      <c r="B22" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="49" t="s">
+        <v>113</v>
+      </c>
+      <c r="G22" s="49"/>
+      <c r="H22" s="49"/>
     </row>
     <row r="23" spans="1:8" ht="76.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B23" s="44" t="s">
-        <v>115</v>
-      </c>
-      <c r="C23" s="44"/>
-      <c r="D23" s="44"/>
-      <c r="E23" s="44"/>
-      <c r="F23" s="45" t="s">
-        <v>123</v>
-      </c>
-      <c r="G23" s="45"/>
-      <c r="H23" s="45"/>
+        <v>68</v>
+      </c>
+      <c r="B23" s="38" t="s">
+        <v>114</v>
+      </c>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+      <c r="F23" s="49" t="s">
+        <v>122</v>
+      </c>
+      <c r="G23" s="49"/>
+      <c r="H23" s="49"/>
     </row>
     <row r="24" spans="1:8" ht="65.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B24" s="44" t="s">
-        <v>124</v>
-      </c>
-      <c r="C24" s="44"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="44"/>
-      <c r="F24" s="45" t="s">
-        <v>126</v>
-      </c>
-      <c r="G24" s="45"/>
-      <c r="H24" s="45"/>
+        <v>49</v>
+      </c>
+      <c r="B24" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="49" t="s">
+        <v>125</v>
+      </c>
+      <c r="G24" s="49"/>
+      <c r="H24" s="49"/>
     </row>
     <row r="25" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B25" s="44" t="s">
-        <v>127</v>
-      </c>
-      <c r="C25" s="44"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="44"/>
-      <c r="F25" s="45" t="s">
-        <v>163</v>
-      </c>
-      <c r="G25" s="45"/>
-      <c r="H25" s="45"/>
+        <v>67</v>
+      </c>
+      <c r="B25" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="G25" s="49"/>
+      <c r="H25" s="49"/>
     </row>
     <row r="26" spans="1:8" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B26" s="43" t="s">
         <v>133</v>
       </c>
-      <c r="B26" s="38" t="s">
-        <v>134</v>
-      </c>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="40"/>
-      <c r="F26" s="41" t="s">
-        <v>164</v>
-      </c>
-      <c r="G26" s="42"/>
-      <c r="H26" s="43"/>
+      <c r="C26" s="44"/>
+      <c r="D26" s="44"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="50" t="s">
+        <v>163</v>
+      </c>
+      <c r="G26" s="51"/>
+      <c r="H26" s="52"/>
     </row>
     <row r="27" spans="1:8" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B27" s="43" t="s">
         <v>140</v>
       </c>
-      <c r="B27" s="38" t="s">
-        <v>141</v>
-      </c>
-      <c r="C27" s="39"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="40"/>
-      <c r="F27" s="41" t="s">
-        <v>165</v>
-      </c>
-      <c r="G27" s="42"/>
-      <c r="H27" s="43"/>
+      <c r="C27" s="44"/>
+      <c r="D27" s="44"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="50" t="s">
+        <v>164</v>
+      </c>
+      <c r="G27" s="51"/>
+      <c r="H27" s="52"/>
     </row>
     <row r="28" spans="1:8" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B28" s="38" t="s">
         <v>150</v>
       </c>
-      <c r="B28" s="44" t="s">
-        <v>151</v>
-      </c>
-      <c r="C28" s="44"/>
-      <c r="D28" s="44"/>
-      <c r="E28" s="44"/>
-      <c r="F28" s="45" t="s">
-        <v>166</v>
-      </c>
-      <c r="G28" s="45"/>
-      <c r="H28" s="45"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="49" t="s">
+        <v>165</v>
+      </c>
+      <c r="G28" s="49"/>
+      <c r="H28" s="49"/>
     </row>
     <row r="29" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="17"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="21"/>
-      <c r="D29" s="21"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="29"/>
-      <c r="G29" s="30"/>
-      <c r="H29" s="31"/>
+      <c r="A29" s="35"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="19"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="18"/>
-      <c r="B30" s="23"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="33"/>
-      <c r="H30" s="34"/>
+      <c r="A30" s="36"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="30"/>
+      <c r="D30" s="30"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="22"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A31" s="18"/>
-      <c r="B31" s="23"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="25"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="33"/>
-      <c r="H31" s="34"/>
+      <c r="A31" s="36"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="30"/>
+      <c r="D31" s="30"/>
+      <c r="E31" s="31"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="22"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A32" s="19"/>
-      <c r="B32" s="26"/>
-      <c r="C32" s="27"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="35"/>
-      <c r="G32" s="36"/>
-      <c r="H32" s="37"/>
+      <c r="A32" s="37"/>
+      <c r="B32" s="32"/>
+      <c r="C32" s="33"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="25"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A33" s="17"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="29"/>
-      <c r="G33" s="30"/>
-      <c r="H33" s="31"/>
+      <c r="A33" s="35"/>
+      <c r="B33" s="26"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="19"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A34" s="18"/>
-      <c r="B34" s="23"/>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="25"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="33"/>
-      <c r="H34" s="34"/>
+      <c r="A34" s="36"/>
+      <c r="B34" s="29"/>
+      <c r="C34" s="30"/>
+      <c r="D34" s="30"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="21"/>
+      <c r="H34" s="22"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A35" s="18"/>
-      <c r="B35" s="23"/>
-      <c r="C35" s="24"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="25"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="33"/>
-      <c r="H35" s="34"/>
+      <c r="A35" s="36"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="30"/>
+      <c r="D35" s="30"/>
+      <c r="E35" s="31"/>
+      <c r="F35" s="20"/>
+      <c r="G35" s="21"/>
+      <c r="H35" s="22"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="19"/>
-      <c r="B36" s="26"/>
-      <c r="C36" s="27"/>
-      <c r="D36" s="27"/>
-      <c r="E36" s="28"/>
-      <c r="F36" s="35"/>
-      <c r="G36" s="36"/>
-      <c r="H36" s="37"/>
+      <c r="A36" s="37"/>
+      <c r="B36" s="32"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="33"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="23"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="25"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="17"/>
-      <c r="B37" s="20"/>
-      <c r="C37" s="21"/>
-      <c r="D37" s="21"/>
-      <c r="E37" s="22"/>
-      <c r="F37" s="29"/>
-      <c r="G37" s="30"/>
-      <c r="H37" s="31"/>
+      <c r="A37" s="35"/>
+      <c r="B37" s="26"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="19"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="18"/>
-      <c r="B38" s="23"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="25"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="33"/>
-      <c r="H38" s="34"/>
+      <c r="A38" s="36"/>
+      <c r="B38" s="29"/>
+      <c r="C38" s="30"/>
+      <c r="D38" s="30"/>
+      <c r="E38" s="31"/>
+      <c r="F38" s="20"/>
+      <c r="G38" s="21"/>
+      <c r="H38" s="22"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" s="18"/>
-      <c r="B39" s="23"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="24"/>
-      <c r="E39" s="25"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="33"/>
-      <c r="H39" s="34"/>
+      <c r="A39" s="36"/>
+      <c r="B39" s="29"/>
+      <c r="C39" s="30"/>
+      <c r="D39" s="30"/>
+      <c r="E39" s="31"/>
+      <c r="F39" s="20"/>
+      <c r="G39" s="21"/>
+      <c r="H39" s="22"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A40" s="19"/>
-      <c r="B40" s="26"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="28"/>
-      <c r="F40" s="35"/>
-      <c r="G40" s="36"/>
-      <c r="H40" s="37"/>
+      <c r="A40" s="37"/>
+      <c r="B40" s="32"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="33"/>
+      <c r="E40" s="34"/>
+      <c r="F40" s="23"/>
+      <c r="G40" s="24"/>
+      <c r="H40" s="25"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A41" s="17"/>
-      <c r="B41" s="20"/>
-      <c r="C41" s="21"/>
-      <c r="D41" s="21"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="29"/>
-      <c r="G41" s="30"/>
-      <c r="H41" s="31"/>
+      <c r="A41" s="35"/>
+      <c r="B41" s="26"/>
+      <c r="C41" s="27"/>
+      <c r="D41" s="27"/>
+      <c r="E41" s="28"/>
+      <c r="F41" s="17"/>
+      <c r="G41" s="18"/>
+      <c r="H41" s="19"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A42" s="18"/>
-      <c r="B42" s="23"/>
-      <c r="C42" s="24"/>
-      <c r="D42" s="24"/>
-      <c r="E42" s="25"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="33"/>
-      <c r="H42" s="34"/>
+      <c r="A42" s="36"/>
+      <c r="B42" s="29"/>
+      <c r="C42" s="30"/>
+      <c r="D42" s="30"/>
+      <c r="E42" s="31"/>
+      <c r="F42" s="20"/>
+      <c r="G42" s="21"/>
+      <c r="H42" s="22"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A43" s="18"/>
-      <c r="B43" s="23"/>
-      <c r="C43" s="24"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="25"/>
-      <c r="F43" s="32"/>
-      <c r="G43" s="33"/>
-      <c r="H43" s="34"/>
+      <c r="A43" s="36"/>
+      <c r="B43" s="29"/>
+      <c r="C43" s="30"/>
+      <c r="D43" s="30"/>
+      <c r="E43" s="31"/>
+      <c r="F43" s="20"/>
+      <c r="G43" s="21"/>
+      <c r="H43" s="22"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A44" s="19"/>
-      <c r="B44" s="26"/>
-      <c r="C44" s="27"/>
-      <c r="D44" s="27"/>
-      <c r="E44" s="28"/>
-      <c r="F44" s="35"/>
-      <c r="G44" s="36"/>
-      <c r="H44" s="37"/>
+      <c r="A44" s="37"/>
+      <c r="B44" s="32"/>
+      <c r="C44" s="33"/>
+      <c r="D44" s="33"/>
+      <c r="E44" s="34"/>
+      <c r="F44" s="23"/>
+      <c r="G44" s="24"/>
+      <c r="H44" s="25"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A45" s="17"/>
-      <c r="B45" s="20"/>
-      <c r="C45" s="21"/>
-      <c r="D45" s="21"/>
-      <c r="E45" s="22"/>
-      <c r="F45" s="29"/>
-      <c r="G45" s="30"/>
-      <c r="H45" s="31"/>
+      <c r="A45" s="35"/>
+      <c r="B45" s="26"/>
+      <c r="C45" s="27"/>
+      <c r="D45" s="27"/>
+      <c r="E45" s="28"/>
+      <c r="F45" s="17"/>
+      <c r="G45" s="18"/>
+      <c r="H45" s="19"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A46" s="18"/>
-      <c r="B46" s="23"/>
-      <c r="C46" s="24"/>
-      <c r="D46" s="24"/>
-      <c r="E46" s="25"/>
-      <c r="F46" s="32"/>
-      <c r="G46" s="33"/>
-      <c r="H46" s="34"/>
+      <c r="A46" s="36"/>
+      <c r="B46" s="29"/>
+      <c r="C46" s="30"/>
+      <c r="D46" s="30"/>
+      <c r="E46" s="31"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="21"/>
+      <c r="H46" s="22"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A47" s="18"/>
-      <c r="B47" s="23"/>
-      <c r="C47" s="24"/>
-      <c r="D47" s="24"/>
-      <c r="E47" s="25"/>
-      <c r="F47" s="32"/>
-      <c r="G47" s="33"/>
-      <c r="H47" s="34"/>
+      <c r="A47" s="36"/>
+      <c r="B47" s="29"/>
+      <c r="C47" s="30"/>
+      <c r="D47" s="30"/>
+      <c r="E47" s="31"/>
+      <c r="F47" s="20"/>
+      <c r="G47" s="21"/>
+      <c r="H47" s="22"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A48" s="19"/>
-      <c r="B48" s="26"/>
-      <c r="C48" s="27"/>
-      <c r="D48" s="27"/>
-      <c r="E48" s="28"/>
-      <c r="F48" s="35"/>
-      <c r="G48" s="36"/>
-      <c r="H48" s="37"/>
+      <c r="A48" s="37"/>
+      <c r="B48" s="32"/>
+      <c r="C48" s="33"/>
+      <c r="D48" s="33"/>
+      <c r="E48" s="34"/>
+      <c r="F48" s="23"/>
+      <c r="G48" s="24"/>
+      <c r="H48" s="25"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A49" s="17"/>
-      <c r="B49" s="20"/>
-      <c r="C49" s="21"/>
-      <c r="D49" s="21"/>
-      <c r="E49" s="22"/>
-      <c r="F49" s="29"/>
-      <c r="G49" s="30"/>
-      <c r="H49" s="31"/>
+      <c r="A49" s="35"/>
+      <c r="B49" s="26"/>
+      <c r="C49" s="27"/>
+      <c r="D49" s="27"/>
+      <c r="E49" s="28"/>
+      <c r="F49" s="17"/>
+      <c r="G49" s="18"/>
+      <c r="H49" s="19"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A50" s="18"/>
-      <c r="B50" s="23"/>
-      <c r="C50" s="24"/>
-      <c r="D50" s="24"/>
-      <c r="E50" s="25"/>
-      <c r="F50" s="32"/>
-      <c r="G50" s="33"/>
-      <c r="H50" s="34"/>
+      <c r="A50" s="36"/>
+      <c r="B50" s="29"/>
+      <c r="C50" s="30"/>
+      <c r="D50" s="30"/>
+      <c r="E50" s="31"/>
+      <c r="F50" s="20"/>
+      <c r="G50" s="21"/>
+      <c r="H50" s="22"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A51" s="18"/>
-      <c r="B51" s="23"/>
-      <c r="C51" s="24"/>
-      <c r="D51" s="24"/>
-      <c r="E51" s="25"/>
-      <c r="F51" s="32"/>
-      <c r="G51" s="33"/>
-      <c r="H51" s="34"/>
+      <c r="A51" s="36"/>
+      <c r="B51" s="29"/>
+      <c r="C51" s="30"/>
+      <c r="D51" s="30"/>
+      <c r="E51" s="31"/>
+      <c r="F51" s="20"/>
+      <c r="G51" s="21"/>
+      <c r="H51" s="22"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A52" s="19"/>
-      <c r="B52" s="26"/>
-      <c r="C52" s="27"/>
-      <c r="D52" s="27"/>
-      <c r="E52" s="28"/>
-      <c r="F52" s="35"/>
-      <c r="G52" s="36"/>
-      <c r="H52" s="37"/>
+      <c r="A52" s="37"/>
+      <c r="B52" s="32"/>
+      <c r="C52" s="33"/>
+      <c r="D52" s="33"/>
+      <c r="E52" s="34"/>
+      <c r="F52" s="23"/>
+      <c r="G52" s="24"/>
+      <c r="H52" s="25"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A53" s="17"/>
-      <c r="B53" s="20"/>
-      <c r="C53" s="21"/>
-      <c r="D53" s="21"/>
-      <c r="E53" s="22"/>
-      <c r="F53" s="29"/>
-      <c r="G53" s="30"/>
-      <c r="H53" s="31"/>
+      <c r="A53" s="35"/>
+      <c r="B53" s="26"/>
+      <c r="C53" s="27"/>
+      <c r="D53" s="27"/>
+      <c r="E53" s="28"/>
+      <c r="F53" s="17"/>
+      <c r="G53" s="18"/>
+      <c r="H53" s="19"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A54" s="18"/>
-      <c r="B54" s="23"/>
-      <c r="C54" s="24"/>
-      <c r="D54" s="24"/>
-      <c r="E54" s="25"/>
-      <c r="F54" s="32"/>
-      <c r="G54" s="33"/>
-      <c r="H54" s="34"/>
+      <c r="A54" s="36"/>
+      <c r="B54" s="29"/>
+      <c r="C54" s="30"/>
+      <c r="D54" s="30"/>
+      <c r="E54" s="31"/>
+      <c r="F54" s="20"/>
+      <c r="G54" s="21"/>
+      <c r="H54" s="22"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A55" s="18"/>
-      <c r="B55" s="23"/>
-      <c r="C55" s="24"/>
-      <c r="D55" s="24"/>
-      <c r="E55" s="25"/>
-      <c r="F55" s="32"/>
-      <c r="G55" s="33"/>
-      <c r="H55" s="34"/>
+      <c r="A55" s="36"/>
+      <c r="B55" s="29"/>
+      <c r="C55" s="30"/>
+      <c r="D55" s="30"/>
+      <c r="E55" s="31"/>
+      <c r="F55" s="20"/>
+      <c r="G55" s="21"/>
+      <c r="H55" s="22"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A56" s="19"/>
-      <c r="B56" s="26"/>
-      <c r="C56" s="27"/>
-      <c r="D56" s="27"/>
-      <c r="E56" s="28"/>
-      <c r="F56" s="35"/>
-      <c r="G56" s="36"/>
-      <c r="H56" s="37"/>
+      <c r="A56" s="37"/>
+      <c r="B56" s="32"/>
+      <c r="C56" s="33"/>
+      <c r="D56" s="33"/>
+      <c r="E56" s="34"/>
+      <c r="F56" s="23"/>
+      <c r="G56" s="24"/>
+      <c r="H56" s="25"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A57" s="17"/>
-      <c r="B57" s="20"/>
-      <c r="C57" s="21"/>
-      <c r="D57" s="21"/>
-      <c r="E57" s="22"/>
-      <c r="F57" s="29"/>
-      <c r="G57" s="30"/>
-      <c r="H57" s="31"/>
+      <c r="A57" s="35"/>
+      <c r="B57" s="26"/>
+      <c r="C57" s="27"/>
+      <c r="D57" s="27"/>
+      <c r="E57" s="28"/>
+      <c r="F57" s="17"/>
+      <c r="G57" s="18"/>
+      <c r="H57" s="19"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A58" s="18"/>
-      <c r="B58" s="23"/>
-      <c r="C58" s="24"/>
-      <c r="D58" s="24"/>
-      <c r="E58" s="25"/>
-      <c r="F58" s="32"/>
-      <c r="G58" s="33"/>
-      <c r="H58" s="34"/>
+      <c r="A58" s="36"/>
+      <c r="B58" s="29"/>
+      <c r="C58" s="30"/>
+      <c r="D58" s="30"/>
+      <c r="E58" s="31"/>
+      <c r="F58" s="20"/>
+      <c r="G58" s="21"/>
+      <c r="H58" s="22"/>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A59" s="18"/>
-      <c r="B59" s="23"/>
-      <c r="C59" s="24"/>
-      <c r="D59" s="24"/>
-      <c r="E59" s="25"/>
-      <c r="F59" s="32"/>
-      <c r="G59" s="33"/>
-      <c r="H59" s="34"/>
+      <c r="A59" s="36"/>
+      <c r="B59" s="29"/>
+      <c r="C59" s="30"/>
+      <c r="D59" s="30"/>
+      <c r="E59" s="31"/>
+      <c r="F59" s="20"/>
+      <c r="G59" s="21"/>
+      <c r="H59" s="22"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A60" s="19"/>
-      <c r="B60" s="26"/>
-      <c r="C60" s="27"/>
-      <c r="D60" s="27"/>
-      <c r="E60" s="28"/>
-      <c r="F60" s="35"/>
-      <c r="G60" s="36"/>
-      <c r="H60" s="37"/>
+      <c r="A60" s="37"/>
+      <c r="B60" s="32"/>
+      <c r="C60" s="33"/>
+      <c r="D60" s="33"/>
+      <c r="E60" s="34"/>
+      <c r="F60" s="23"/>
+      <c r="G60" s="24"/>
+      <c r="H60" s="25"/>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A61" s="17"/>
-      <c r="B61" s="20"/>
-      <c r="C61" s="21"/>
-      <c r="D61" s="21"/>
-      <c r="E61" s="22"/>
-      <c r="F61" s="29"/>
-      <c r="G61" s="30"/>
-      <c r="H61" s="31"/>
+      <c r="A61" s="35"/>
+      <c r="B61" s="26"/>
+      <c r="C61" s="27"/>
+      <c r="D61" s="27"/>
+      <c r="E61" s="28"/>
+      <c r="F61" s="17"/>
+      <c r="G61" s="18"/>
+      <c r="H61" s="19"/>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A62" s="18"/>
-      <c r="B62" s="23"/>
-      <c r="C62" s="24"/>
-      <c r="D62" s="24"/>
-      <c r="E62" s="25"/>
-      <c r="F62" s="32"/>
-      <c r="G62" s="33"/>
-      <c r="H62" s="34"/>
+      <c r="A62" s="36"/>
+      <c r="B62" s="29"/>
+      <c r="C62" s="30"/>
+      <c r="D62" s="30"/>
+      <c r="E62" s="31"/>
+      <c r="F62" s="20"/>
+      <c r="G62" s="21"/>
+      <c r="H62" s="22"/>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A63" s="18"/>
-      <c r="B63" s="23"/>
-      <c r="C63" s="24"/>
-      <c r="D63" s="24"/>
-      <c r="E63" s="25"/>
-      <c r="F63" s="32"/>
-      <c r="G63" s="33"/>
-      <c r="H63" s="34"/>
+      <c r="A63" s="36"/>
+      <c r="B63" s="29"/>
+      <c r="C63" s="30"/>
+      <c r="D63" s="30"/>
+      <c r="E63" s="31"/>
+      <c r="F63" s="20"/>
+      <c r="G63" s="21"/>
+      <c r="H63" s="22"/>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A64" s="19"/>
-      <c r="B64" s="26"/>
-      <c r="C64" s="27"/>
-      <c r="D64" s="27"/>
-      <c r="E64" s="28"/>
-      <c r="F64" s="35"/>
-      <c r="G64" s="36"/>
-      <c r="H64" s="37"/>
+      <c r="A64" s="37"/>
+      <c r="B64" s="32"/>
+      <c r="C64" s="33"/>
+      <c r="D64" s="33"/>
+      <c r="E64" s="34"/>
+      <c r="F64" s="23"/>
+      <c r="G64" s="24"/>
+      <c r="H64" s="25"/>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A65" s="17"/>
-      <c r="B65" s="20"/>
-      <c r="C65" s="21"/>
-      <c r="D65" s="21"/>
-      <c r="E65" s="22"/>
-      <c r="F65" s="29"/>
-      <c r="G65" s="30"/>
-      <c r="H65" s="31"/>
+      <c r="A65" s="35"/>
+      <c r="B65" s="26"/>
+      <c r="C65" s="27"/>
+      <c r="D65" s="27"/>
+      <c r="E65" s="28"/>
+      <c r="F65" s="17"/>
+      <c r="G65" s="18"/>
+      <c r="H65" s="19"/>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A66" s="18"/>
-      <c r="B66" s="23"/>
-      <c r="C66" s="24"/>
-      <c r="D66" s="24"/>
-      <c r="E66" s="25"/>
-      <c r="F66" s="32"/>
-      <c r="G66" s="33"/>
-      <c r="H66" s="34"/>
+      <c r="A66" s="36"/>
+      <c r="B66" s="29"/>
+      <c r="C66" s="30"/>
+      <c r="D66" s="30"/>
+      <c r="E66" s="31"/>
+      <c r="F66" s="20"/>
+      <c r="G66" s="21"/>
+      <c r="H66" s="22"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A67" s="18"/>
-      <c r="B67" s="23"/>
-      <c r="C67" s="24"/>
-      <c r="D67" s="24"/>
-      <c r="E67" s="25"/>
-      <c r="F67" s="32"/>
-      <c r="G67" s="33"/>
-      <c r="H67" s="34"/>
+      <c r="A67" s="36"/>
+      <c r="B67" s="29"/>
+      <c r="C67" s="30"/>
+      <c r="D67" s="30"/>
+      <c r="E67" s="31"/>
+      <c r="F67" s="20"/>
+      <c r="G67" s="21"/>
+      <c r="H67" s="22"/>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A68" s="19"/>
-      <c r="B68" s="26"/>
-      <c r="C68" s="27"/>
-      <c r="D68" s="27"/>
-      <c r="E68" s="28"/>
-      <c r="F68" s="35"/>
-      <c r="G68" s="36"/>
-      <c r="H68" s="37"/>
+      <c r="A68" s="37"/>
+      <c r="B68" s="32"/>
+      <c r="C68" s="33"/>
+      <c r="D68" s="33"/>
+      <c r="E68" s="34"/>
+      <c r="F68" s="23"/>
+      <c r="G68" s="24"/>
+      <c r="H68" s="25"/>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A69" s="17"/>
-      <c r="B69" s="20"/>
-      <c r="C69" s="21"/>
-      <c r="D69" s="21"/>
-      <c r="E69" s="22"/>
-      <c r="F69" s="29"/>
-      <c r="G69" s="30"/>
-      <c r="H69" s="31"/>
+      <c r="A69" s="35"/>
+      <c r="B69" s="26"/>
+      <c r="C69" s="27"/>
+      <c r="D69" s="27"/>
+      <c r="E69" s="28"/>
+      <c r="F69" s="17"/>
+      <c r="G69" s="18"/>
+      <c r="H69" s="19"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A70" s="18"/>
-      <c r="B70" s="23"/>
-      <c r="C70" s="24"/>
-      <c r="D70" s="24"/>
-      <c r="E70" s="25"/>
-      <c r="F70" s="32"/>
-      <c r="G70" s="33"/>
-      <c r="H70" s="34"/>
+      <c r="A70" s="36"/>
+      <c r="B70" s="29"/>
+      <c r="C70" s="30"/>
+      <c r="D70" s="30"/>
+      <c r="E70" s="31"/>
+      <c r="F70" s="20"/>
+      <c r="G70" s="21"/>
+      <c r="H70" s="22"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A71" s="18"/>
-      <c r="B71" s="23"/>
-      <c r="C71" s="24"/>
-      <c r="D71" s="24"/>
-      <c r="E71" s="25"/>
-      <c r="F71" s="32"/>
-      <c r="G71" s="33"/>
-      <c r="H71" s="34"/>
+      <c r="A71" s="36"/>
+      <c r="B71" s="29"/>
+      <c r="C71" s="30"/>
+      <c r="D71" s="30"/>
+      <c r="E71" s="31"/>
+      <c r="F71" s="20"/>
+      <c r="G71" s="21"/>
+      <c r="H71" s="22"/>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A72" s="19"/>
-      <c r="B72" s="26"/>
-      <c r="C72" s="27"/>
-      <c r="D72" s="27"/>
-      <c r="E72" s="28"/>
-      <c r="F72" s="35"/>
-      <c r="G72" s="36"/>
-      <c r="H72" s="37"/>
+      <c r="A72" s="37"/>
+      <c r="B72" s="32"/>
+      <c r="C72" s="33"/>
+      <c r="D72" s="33"/>
+      <c r="E72" s="34"/>
+      <c r="F72" s="23"/>
+      <c r="G72" s="24"/>
+      <c r="H72" s="25"/>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A73" s="17"/>
-      <c r="B73" s="20"/>
-      <c r="C73" s="21"/>
-      <c r="D73" s="21"/>
-      <c r="E73" s="22"/>
-      <c r="F73" s="29"/>
-      <c r="G73" s="30"/>
-      <c r="H73" s="31"/>
+      <c r="A73" s="35"/>
+      <c r="B73" s="26"/>
+      <c r="C73" s="27"/>
+      <c r="D73" s="27"/>
+      <c r="E73" s="28"/>
+      <c r="F73" s="17"/>
+      <c r="G73" s="18"/>
+      <c r="H73" s="19"/>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A74" s="18"/>
-      <c r="B74" s="23"/>
-      <c r="C74" s="24"/>
-      <c r="D74" s="24"/>
-      <c r="E74" s="25"/>
-      <c r="F74" s="32"/>
-      <c r="G74" s="33"/>
-      <c r="H74" s="34"/>
+      <c r="A74" s="36"/>
+      <c r="B74" s="29"/>
+      <c r="C74" s="30"/>
+      <c r="D74" s="30"/>
+      <c r="E74" s="31"/>
+      <c r="F74" s="20"/>
+      <c r="G74" s="21"/>
+      <c r="H74" s="22"/>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A75" s="18"/>
-      <c r="B75" s="23"/>
-      <c r="C75" s="24"/>
-      <c r="D75" s="24"/>
-      <c r="E75" s="25"/>
-      <c r="F75" s="32"/>
-      <c r="G75" s="33"/>
-      <c r="H75" s="34"/>
+      <c r="A75" s="36"/>
+      <c r="B75" s="29"/>
+      <c r="C75" s="30"/>
+      <c r="D75" s="30"/>
+      <c r="E75" s="31"/>
+      <c r="F75" s="20"/>
+      <c r="G75" s="21"/>
+      <c r="H75" s="22"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A76" s="19"/>
-      <c r="B76" s="26"/>
-      <c r="C76" s="27"/>
-      <c r="D76" s="27"/>
-      <c r="E76" s="28"/>
-      <c r="F76" s="35"/>
-      <c r="G76" s="36"/>
-      <c r="H76" s="37"/>
+      <c r="A76" s="37"/>
+      <c r="B76" s="32"/>
+      <c r="C76" s="33"/>
+      <c r="D76" s="33"/>
+      <c r="E76" s="34"/>
+      <c r="F76" s="23"/>
+      <c r="G76" s="24"/>
+      <c r="H76" s="25"/>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A77" s="17"/>
-      <c r="B77" s="20"/>
-      <c r="C77" s="21"/>
-      <c r="D77" s="21"/>
-      <c r="E77" s="22"/>
-      <c r="F77" s="29"/>
-      <c r="G77" s="30"/>
-      <c r="H77" s="31"/>
+      <c r="A77" s="35"/>
+      <c r="B77" s="26"/>
+      <c r="C77" s="27"/>
+      <c r="D77" s="27"/>
+      <c r="E77" s="28"/>
+      <c r="F77" s="17"/>
+      <c r="G77" s="18"/>
+      <c r="H77" s="19"/>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A78" s="18"/>
-      <c r="B78" s="23"/>
-      <c r="C78" s="24"/>
-      <c r="D78" s="24"/>
-      <c r="E78" s="25"/>
-      <c r="F78" s="32"/>
-      <c r="G78" s="33"/>
-      <c r="H78" s="34"/>
+      <c r="A78" s="36"/>
+      <c r="B78" s="29"/>
+      <c r="C78" s="30"/>
+      <c r="D78" s="30"/>
+      <c r="E78" s="31"/>
+      <c r="F78" s="20"/>
+      <c r="G78" s="21"/>
+      <c r="H78" s="22"/>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A79" s="18"/>
-      <c r="B79" s="23"/>
-      <c r="C79" s="24"/>
-      <c r="D79" s="24"/>
-      <c r="E79" s="25"/>
-      <c r="F79" s="32"/>
-      <c r="G79" s="33"/>
-      <c r="H79" s="34"/>
+      <c r="A79" s="36"/>
+      <c r="B79" s="29"/>
+      <c r="C79" s="30"/>
+      <c r="D79" s="30"/>
+      <c r="E79" s="31"/>
+      <c r="F79" s="20"/>
+      <c r="G79" s="21"/>
+      <c r="H79" s="22"/>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A80" s="19"/>
-      <c r="B80" s="26"/>
-      <c r="C80" s="27"/>
-      <c r="D80" s="27"/>
-      <c r="E80" s="28"/>
-      <c r="F80" s="35"/>
-      <c r="G80" s="36"/>
-      <c r="H80" s="37"/>
+      <c r="A80" s="37"/>
+      <c r="B80" s="32"/>
+      <c r="C80" s="33"/>
+      <c r="D80" s="33"/>
+      <c r="E80" s="34"/>
+      <c r="F80" s="23"/>
+      <c r="G80" s="24"/>
+      <c r="H80" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="79">
+    <mergeCell ref="A61:A64"/>
+    <mergeCell ref="B61:E64"/>
+    <mergeCell ref="F61:H64"/>
+    <mergeCell ref="F53:H56"/>
+    <mergeCell ref="B53:E56"/>
+    <mergeCell ref="A53:A56"/>
+    <mergeCell ref="A57:A60"/>
+    <mergeCell ref="B57:E60"/>
+    <mergeCell ref="F57:H60"/>
+    <mergeCell ref="F45:H48"/>
+    <mergeCell ref="B45:E48"/>
+    <mergeCell ref="A45:A48"/>
+    <mergeCell ref="A49:A52"/>
+    <mergeCell ref="B49:E52"/>
+    <mergeCell ref="F49:H52"/>
+    <mergeCell ref="A37:A40"/>
+    <mergeCell ref="B37:E40"/>
+    <mergeCell ref="F37:H40"/>
+    <mergeCell ref="F41:H44"/>
+    <mergeCell ref="B41:E44"/>
+    <mergeCell ref="A41:A44"/>
+    <mergeCell ref="A29:A32"/>
+    <mergeCell ref="B29:E32"/>
+    <mergeCell ref="F29:H32"/>
+    <mergeCell ref="A33:A36"/>
+    <mergeCell ref="B33:E36"/>
+    <mergeCell ref="F33:H36"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="F24:H24"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="F25:H25"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B11:H11"/>
     <mergeCell ref="F65:H68"/>
     <mergeCell ref="B73:E76"/>
     <mergeCell ref="F69:H72"/>
@@ -2510,73 +2577,6 @@
     <mergeCell ref="A69:A72"/>
     <mergeCell ref="B69:E72"/>
     <mergeCell ref="A73:A76"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B15:H15"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="F21:H21"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="F18:H18"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="B20:E20"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="F24:H24"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="F25:H25"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="F26:H26"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="F27:H27"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="F28:H28"/>
-    <mergeCell ref="A29:A32"/>
-    <mergeCell ref="B29:E32"/>
-    <mergeCell ref="F29:H32"/>
-    <mergeCell ref="A33:A36"/>
-    <mergeCell ref="B33:E36"/>
-    <mergeCell ref="F33:H36"/>
-    <mergeCell ref="A37:A40"/>
-    <mergeCell ref="B37:E40"/>
-    <mergeCell ref="F37:H40"/>
-    <mergeCell ref="F41:H44"/>
-    <mergeCell ref="B41:E44"/>
-    <mergeCell ref="A41:A44"/>
-    <mergeCell ref="F45:H48"/>
-    <mergeCell ref="B45:E48"/>
-    <mergeCell ref="A45:A48"/>
-    <mergeCell ref="A49:A52"/>
-    <mergeCell ref="B49:E52"/>
-    <mergeCell ref="F49:H52"/>
-    <mergeCell ref="A61:A64"/>
-    <mergeCell ref="B61:E64"/>
-    <mergeCell ref="F61:H64"/>
-    <mergeCell ref="F53:H56"/>
-    <mergeCell ref="B53:E56"/>
-    <mergeCell ref="A53:A56"/>
-    <mergeCell ref="A57:A60"/>
-    <mergeCell ref="B57:E60"/>
-    <mergeCell ref="F57:H60"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <hyperlinks>
@@ -2607,16 +2607,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>23</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>24</v>
       </c>
       <c r="E1" s="16" t="s">
         <v>0</v>
@@ -2624,70 +2624,70 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="1">
         <v>25</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -2705,16 +2705,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>23</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>24</v>
       </c>
       <c r="E1" s="16" t="s">
         <v>0</v>
@@ -2722,121 +2722,121 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="1">
         <v>100</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C4" s="1">
         <v>20</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" s="1">
         <v>100</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6" s="1">
         <v>20</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C7" s="1">
         <v>100</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="E8" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -2854,16 +2854,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>23</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>24</v>
       </c>
       <c r="E1" s="16" t="s">
         <v>0</v>
@@ -2871,155 +2871,155 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2" s="1">
         <v>25</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C4" s="1">
         <v>25</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" s="1">
         <v>100</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6" s="1">
         <v>20</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>161</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="E9" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="E10" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -3045,16 +3045,16 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="C1" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="D1" s="12" t="s">
         <v>23</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>24</v>
       </c>
       <c r="E1" s="13" t="s">
         <v>0</v>
@@ -3064,127 +3064,127 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>27</v>
-      </c>
       <c r="E2" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G2" s="7"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="1">
         <v>50</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G3" s="7"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="C4" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="G4" s="7"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" s="1">
         <v>20</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G5" s="7"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6" s="1">
         <v>255</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C7" s="1">
         <v>255</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G7" s="7"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="E8" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G8" s="7"/>
     </row>
@@ -3237,16 +3237,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>23</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>24</v>
       </c>
       <c r="E1" s="16" t="s">
         <v>0</v>
@@ -3254,155 +3254,155 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="16" t="s">
-        <v>27</v>
-      </c>
       <c r="E2" s="16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="1">
         <v>50</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C4" s="1">
         <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" s="1">
         <v>255</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6" s="1">
         <v>255</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C7" s="1">
         <v>20</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C8" s="1">
         <v>100</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="E9" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="E10" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -3420,16 +3420,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>23</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>24</v>
       </c>
       <c r="E1" s="16" t="s">
         <v>0</v>
@@ -3437,36 +3437,36 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2" s="1">
         <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="1">
         <v>100</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -3484,16 +3484,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>23</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>24</v>
       </c>
       <c r="E1" s="16" t="s">
         <v>0</v>
@@ -3501,53 +3501,53 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2" s="1">
         <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="1">
         <v>100</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C4" s="1">
         <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -3565,16 +3565,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>23</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>24</v>
       </c>
       <c r="E1" s="16" t="s">
         <v>0</v>
@@ -3582,53 +3582,53 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="1">
         <v>50</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="E4" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -3646,16 +3646,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="C1" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="D1" s="15" t="s">
         <v>23</v>
-      </c>
-      <c r="D1" s="15" t="s">
-        <v>24</v>
       </c>
       <c r="E1" s="15" t="s">
         <v>0</v>
@@ -3663,87 +3663,87 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="1">
         <v>255</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C4" s="1">
         <v>10.199999999999999</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C5" s="1">
         <v>10.199999999999999</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -3761,16 +3761,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>23</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>24</v>
       </c>
       <c r="E1" s="16" t="s">
         <v>0</v>
@@ -3778,53 +3778,53 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="1">
         <v>50</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="E4" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -3842,16 +3842,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>23</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>24</v>
       </c>
       <c r="E1" s="16" t="s">
         <v>0</v>
@@ -3859,87 +3859,87 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2" s="1">
         <v>25</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="1">
         <v>50</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="E4" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C5" s="1">
         <v>10.199999999999999</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="D6" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>